<commit_message>
Redesign Agent 4: graphic illustrations instead of text slides
- Claude generates full SVG graphics with visual metaphors
- Abstract shapes, flowing lines, constellations, organic curves
- Minimal text: only topic tag pill + small signature
- Fallback template: 20+ geometric elements if Claude fails
- DALL-E prompt extracted from Claude's design intent

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
+++ b/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -124,6 +124,16 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -216,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -316,6 +326,24 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -682,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -694,6 +722,7 @@
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -756,6 +785,11 @@
           <t>סטטוס</t>
         </is>
       </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>🖼️ תמונה מצורפת</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
@@ -802,6 +836,11 @@
       <c r="I4" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J4" s="34" t="inlineStr">
+        <is>
+          <t>פרק_01_שייכות_ומדידה_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -843,6 +882,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J5" s="35" t="inlineStr">
+        <is>
+          <t>פרק_01_שייכות_ומדידה_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="11" t="inlineStr"/>
@@ -882,6 +926,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J6" s="36" t="inlineStr">
+        <is>
+          <t>פרק_01_שייכות_ומדידה_PODCAST.svg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -928,6 +977,11 @@
       <c r="I7" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J7" s="34" t="inlineStr">
+        <is>
+          <t>פרק_02_תקווה_בחירום_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -969,6 +1023,11 @@
           <t>⚠️ לבחור גרסה</t>
         </is>
       </c>
+      <c r="J8" s="37" t="inlineStr">
+        <is>
+          <t>פרק_02_תקווה_בחירום_BLOG.svg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="11" t="inlineStr"/>
@@ -1008,6 +1067,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J9" s="35" t="inlineStr">
+        <is>
+          <t>פרק_02_תקווה_בחירום_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="11" t="inlineStr"/>
@@ -1043,6 +1107,11 @@
           <t>❌ חסר</t>
         </is>
       </c>
+      <c r="J10" s="38" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב לפודקאסט</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -1089,6 +1158,11 @@
       <c r="I11" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>פרק_03_מרחב_שמשנה_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -1126,6 +1200,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>פרק_03_מרחב_שמשנה_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="11" t="inlineStr"/>
@@ -1161,6 +1240,11 @@
           <t>❌ חסר</t>
         </is>
       </c>
+      <c r="J13" s="38" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב לפודקאסט</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -1207,6 +1291,11 @@
       <c r="I14" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>פרק_04_נוער_דיגיטלי_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -1244,6 +1333,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J15" s="35" t="inlineStr">
+        <is>
+          <t>פרק_04_נוער_דיגיטלי_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="11" t="inlineStr"/>
@@ -1283,6 +1377,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J16" s="36" t="inlineStr">
+        <is>
+          <t>פרק_04_נוער_דיגיטלי_PODCAST.svg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -1329,6 +1428,11 @@
       <c r="I17" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J17" s="34" t="inlineStr">
+        <is>
+          <t>פרק_05_מעברים_וסף_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -1366,6 +1470,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J18" s="35" t="inlineStr">
+        <is>
+          <t>פרק_05_מעברים_וסף_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="11" t="inlineStr"/>
@@ -1401,6 +1510,11 @@
           <t>❌ חסר</t>
         </is>
       </c>
+      <c r="J19" s="38" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב לפודקאסט</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1447,6 +1561,11 @@
       <c r="I20" s="10" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_BLOG.svg</t>
         </is>
       </c>
     </row>
@@ -1484,6 +1603,11 @@
           <t>✅ מוכן</t>
         </is>
       </c>
+      <c r="J21" s="35" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_LINKEDIN.svg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="11" t="inlineStr"/>
@@ -1521,6 +1645,11 @@
       <c r="I22" s="16" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J22" s="36" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_PODCAST.svg</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2496,6 +2625,20 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>תמונות</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>כל קבצי ה-SVG נמצאים בתיקייה:
+output/designs/
+הקבצים הממוספרים (פרק_01_...) הם הגרסאות הסופיות לפרסום.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Add personal context, rejection learning, and published tracking
memory.py:
- get_context/save_context: personal season, purpose, tensions, questions
- record_published/get_published_titles: prevent content repetition
- save_rejection_rule/get_rejection_rules: learn from rejected content
- format_rules_for_prompt: inject learned rules into prompts

context_update.py:
- Interactive questionnaire (5 dimensions)
- Quick update via claude_cli ("--quick 'מחפש עבודה'")
- Show current context

agent3_content_creator.py:
- System prompt includes personal context + published titles + rejection rules

agent3_5_human_review.py:
- On rejection: extracts a rule via claude_cli and saves to memory
- Rules apply to all future content generation

agent5_project_manager.py:
- New chat command: "קונטקסט" / "context"

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
+++ b/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
@@ -722,7 +722,7 @@
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="J10" s="38" t="inlineStr">
         <is>
-          <t>❌ חסר עיצוב לפודקאסט</t>
+          <t>❌ חסר עיצוב — יש לייצר</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="J13" s="38" t="inlineStr">
         <is>
-          <t>❌ חסר עיצוב לפודקאסט</t>
+          <t>❌ חסר עיצוב — יש לייצר</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="J19" s="38" t="inlineStr">
         <is>
-          <t>❌ חסר עיצוב לפודקאסט</t>
+          <t>❌ חסר עיצוב — יש לייצר</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance writers: APA 7 rules + HE as translation + smart truncation
agent2_writer.py:
- APA 7 citation rules added to system prompt
- HE article now TRANSLATES from EN (not rewrites from scratch)
- Saves ~$1 and 1-2 minutes on bilingual runs

agent3_content_creator.py:
- Smart article truncation: intro + middle + conclusion (saves ~50% tokens)
- Each platform now requires references section (2-6 sources APA 7)
- LinkedIn: sources at bottom
- Blog: inline citations + full references section
- Podcast: spoken citations + show notes with references

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
+++ b/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -134,6 +134,33 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002E75B6"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -226,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -343,6 +370,54 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -710,7 +785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1555,12 +1630,12 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>פוסט סיום מאתגר — הטיעון המרכזי של הסדרה</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>✅ מוכן</t>
+          <t>⚠️ קיימת גרסה חדשה — v2 (2007). לבחור לפני פרסום</t>
+        </is>
+      </c>
+      <c r="I20" s="40" t="inlineStr">
+        <is>
+          <t>⚠️ לבחור גרסה</t>
         </is>
       </c>
       <c r="J20" s="34" t="inlineStr">
@@ -1650,6 +1725,183 @@
       <c r="J22" s="36" t="inlineStr">
         <is>
           <t>פרק_06_ביקורת_מערכתית_PODCAST.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="41" t="inlineStr"/>
+      <c r="B23" s="12" t="inlineStr"/>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>📝 בלוג v2</t>
+        </is>
+      </c>
+      <c r="D23" s="43" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_BLOG_v2.md</t>
+        </is>
+      </c>
+      <c r="E23" s="43" t="inlineStr">
+        <is>
+          <t>החינוך הבלתי פורמלי לא בנוי לפצות — הוא בנוי להכיל</t>
+        </is>
+      </c>
+      <c r="F23" s="42" t="inlineStr">
+        <is>
+          <t>שבוע 6</t>
+        </is>
+      </c>
+      <c r="G23" s="43" t="inlineStr">
+        <is>
+          <t>הכלה, סוכנות אזרחית, נוער בסיכון, מחנכים</t>
+        </is>
+      </c>
+      <c r="H23" s="43" t="inlineStr">
+        <is>
+          <t>גרסה חדשה יותר (20:07). לבחור בין v1 ל-v2 לפני פרסום</t>
+        </is>
+      </c>
+      <c r="I23" s="44" t="inlineStr">
+        <is>
+          <t>⚠️ לבחור גרסה</t>
+        </is>
+      </c>
+      <c r="J23" s="45" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_BLOG_v2.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="46" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>המבנה הוא המסר
+ראובן כהנא</t>
+        </is>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>📝 בלוג</t>
+        </is>
+      </c>
+      <c r="D24" s="48" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_BLOG.md</t>
+        </is>
+      </c>
+      <c r="E24" s="48" t="inlineStr">
+        <is>
+          <t>המבנה הוא המסר: מה שבית הספר לא יכול לעשות — ולמה</t>
+        </is>
+      </c>
+      <c r="F24" s="47" t="inlineStr">
+        <is>
+          <t>שבוע 7</t>
+        </is>
+      </c>
+      <c r="G24" s="48" t="inlineStr">
+        <is>
+          <t>ראובן כהנא, תנועות נוער, מבנה ותוכן, זהות, מדריכים</t>
+        </is>
+      </c>
+      <c r="H24" s="48" t="inlineStr">
+        <is>
+          <t>פרק חדש! על תיאוריית כהנא — המבנה מאפשר זהות</t>
+        </is>
+      </c>
+      <c r="I24" s="49" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J24" s="50" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_BLOG.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="41" t="inlineStr"/>
+      <c r="B25" s="12" t="inlineStr"/>
+      <c r="C25" s="42" t="inlineStr">
+        <is>
+          <t>💼 לינקדאין</t>
+        </is>
+      </c>
+      <c r="D25" s="43" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_LINKEDIN.txt</t>
+        </is>
+      </c>
+      <c r="E25" s="43" t="inlineStr">
+        <is>
+          <t>("קהאנה כתב שמה שמייחד את החינוך הבלתי פורמלי הוא לא התוכן — זה המבנה")</t>
+        </is>
+      </c>
+      <c r="F25" s="42" t="inlineStr">
+        <is>
+          <t>שבוע 7</t>
+        </is>
+      </c>
+      <c r="G25" s="43" t="inlineStr">
+        <is>
+          <t>כהנא, מבנה, חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="H25" s="43" t="inlineStr"/>
+      <c r="I25" s="51" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J25" s="45" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_LINKEDIN.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="41" t="inlineStr"/>
+      <c r="B26" s="12" t="inlineStr"/>
+      <c r="C26" s="52" t="inlineStr">
+        <is>
+          <t>🎙️ פודקאסט</t>
+        </is>
+      </c>
+      <c r="D26" s="53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="53" t="inlineStr">
+        <is>
+          <t>פרק 7: עדיין לא נוצר</t>
+        </is>
+      </c>
+      <c r="F26" s="52" t="inlineStr">
+        <is>
+          <t>שבוע 7</t>
+        </is>
+      </c>
+      <c r="G26" s="53" t="inlineStr"/>
+      <c r="H26" s="53" t="inlineStr">
+        <is>
+          <t>❌ חסר סקריפט — יש לייצר</t>
+        </is>
+      </c>
+      <c r="I26" s="54" t="inlineStr">
+        <is>
+          <t>❌ חסר</t>
+        </is>
+      </c>
+      <c r="J26" s="55" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוד</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2473,6 +2725,182 @@
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_BLOG_v2.md</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>פרק 6 v2 — ביקורת</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה חדשה</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>לבחור בין v1 ל-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_BLOG.md</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>פרק 7 — כהנא</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>✅ סופי</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>פרק חדש</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_LINKEDIN.txt</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>פרק 7 — כהנא</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>✅ סופי</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_BLOG_v2.svg</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>פרק 6 — עיצוב v2</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה חדשה</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_BLOG.svg</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>פרק 7 — עיצוב</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E33" s="25" t="inlineStr">
+        <is>
+          <t>✅ סופי</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>פרק_07_המבנה_הוא_המסר_LINKEDIN.svg</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>פרק 7 — עיצוב LI</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>✅ סופי</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Address code review feedback: revert 4 over-engineered features
1. Revert forced "always 3 platforms" — back to smart default that
   classifier can override. Not every topic needs a podcast.
2. Remove colored diff in Agent 3.5 — unnecessary curses-like
   complexity for a terminal tool. Back to simple "file updated" display.
3. Remove brand consistency auto-inject in Agent 4 — the prompt
   already specifies colors. Injecting style= on the SVG tag is
   not meaningful brand validation.
4. Rename test_chat_smoke → test_chat_audit — it's an architecture
   audit (import + runtime path check), not an end-to-end smoke test.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
+++ b/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -161,8 +161,17 @@
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -234,6 +243,30 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+        <bgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -253,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -420,6 +453,22 @@
     <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -785,19 +834,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -808,9 +857,9 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>פז שלמה | 2026  |  6 פרקים × 3 פלטפורמות</t>
+      <c r="A2" s="59" t="inlineStr">
+        <is>
+          <t>פז שלמה | 2026  |  8 פרקים × 3 פלטפורמות</t>
         </is>
       </c>
     </row>
@@ -867,53 +916,53 @@
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>שייכות ומדידה
 מה שבניתי לא נמדד</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="61" t="inlineStr">
         <is>
           <t>youth_movements_x_peer_mentorship_x_assessment_and_en_blog_20260407_1322.md</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="61" t="inlineStr">
         <is>
           <t>מה שבניתי לא נמדד — ולכן, לכאורה, לא קרה</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="61" t="inlineStr">
         <is>
           <t>שבוע 1</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="61" t="inlineStr">
         <is>
           <t>שייכות, מדריכים, תנועות נוער, מדידת השפעה</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="61" t="inlineStr">
         <is>
           <t>פוסט פתיחה — מציג את הפרדוקס המרכזי</t>
         </is>
       </c>
-      <c r="I4" s="10" t="inlineStr">
+      <c r="I4" s="60" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J4" s="34" t="inlineStr">
+      <c r="J4" s="61" t="inlineStr">
         <is>
           <t>פרק_01_שייכות_ומדידה_BLOG.svg</t>
         </is>
@@ -1008,53 +1057,53 @@
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="61" t="inlineStr">
         <is>
           <t>תקווה בחירום
 כשבית הספר נשבר</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="61" t="inlineStr">
         <is>
           <t>education_durin_x_education_for_h_x_non-formal_edu_en_blog_20260407_1148.md</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>כשבית הספר נשבר — מי מחזיק את התקווה?</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="61" t="inlineStr">
         <is>
           <t>שבוע 2</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="61" t="inlineStr">
         <is>
           <t>תקווה, חוסן נפשי, שייכות, חינוך בחירום</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="61" t="inlineStr">
         <is>
           <t>גרסה א׳ — זווית: תקווה ושייכות</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I7" s="60" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J7" s="34" t="inlineStr">
+      <c r="J7" s="61" t="inlineStr">
         <is>
           <t>פרק_02_תקווה_בחירום_BLOG.svg</t>
         </is>
@@ -1158,7 +1207,7 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>education_for_hope_en_podcast_script_20260407_1028.md</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -1174,12 +1223,12 @@
       <c r="G10" s="15" t="inlineStr"/>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>❌ חסר סקריפט — יש לייצר</t>
+          <t>⚠️ גרסה מוקדמת — מ-posts/ root, לבדוק אם מתאים לסדרה</t>
         </is>
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>❌ חסר</t>
+          <t>⚠️ לבדיקה</t>
         </is>
       </c>
       <c r="J10" s="38" t="inlineStr">
@@ -1189,53 +1238,53 @@
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="60" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>מרחב שמשנה
 לא הייתי המחנך הטוב</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="61" t="inlineStr">
         <is>
           <t>outdoor_and_adv_x_arts-based_non-_x_digital_youth__en_blog_20260407_2246.md</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>לא הייתי המחנך הטוב — הייתי רק שם כשהמרחב עשה את העבודה</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="61" t="inlineStr">
         <is>
           <t>שבוע 3</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="61" t="inlineStr">
         <is>
           <t>חוץ ואתגר, אומנות, מרחב חינוכי, זהות</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H11" s="61" t="inlineStr">
         <is>
           <t>פוסט עם פתיחה סיפורית חזקה (ת. שלא דיבר)</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="60" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J11" s="34" t="inlineStr">
+      <c r="J11" s="61" t="inlineStr">
         <is>
           <t>פרק_03_מרחב_שמשנה_BLOG.svg</t>
         </is>
@@ -1307,7 +1356,7 @@
       <c r="G13" s="15" t="inlineStr"/>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>❌ חסר סקריפט — יש לייצר</t>
+          <t>❌ חסר סקריפט — יש לייצר (גרסת outdoor קיימת ב-articles)</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
@@ -1322,53 +1371,53 @@
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="60" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="61" t="inlineStr">
         <is>
           <t>נוער דיגיטלי
 מה קורה כשנער מרים מצלמה</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="61" t="inlineStr">
         <is>
           <t>digital_youth_w_x_digital_youth_w_x_arts-based_non_en_blog_20260408_1242.md</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="61" t="inlineStr">
         <is>
           <t>מה קורה כשנער מרים מצלמה ולא יודע שהוא מגדיר את עצמו?</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="61" t="inlineStr">
         <is>
           <t>שבוע 4</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="61" t="inlineStr">
         <is>
           <t>יצירה דיגיטלית, זהות, אוריינות מדיה, מדריכים</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="61" t="inlineStr">
         <is>
           <t>הגרסה הסופית (v2 מ-08/04). לא להשתמש ב-2359 של 07/04</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="I14" s="60" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J14" s="34" t="inlineStr">
+      <c r="J14" s="61" t="inlineStr">
         <is>
           <t>פרק_04_נוער_דיגיטלי_BLOG.svg</t>
         </is>
@@ -1459,53 +1508,53 @@
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="60" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>מעברים וסף
 הסף הוא לא שלב — הוא מקום</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="61" t="inlineStr">
         <is>
           <t>new_beginnings__x_fresh_start_eff_x_threshold_conc_en_blog_20260407_1741.md</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="61" t="inlineStr">
         <is>
           <t>הסף הוא לא שלב — הוא מקום</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="61" t="inlineStr">
         <is>
           <t>שבוע 5</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="61" t="inlineStr">
         <is>
           <t>מעברים, לימינליות, זהות, שייכות, בסיס בטוח</t>
         </is>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H17" s="61" t="inlineStr">
         <is>
           <t>פוסט עמוק על הרגע שבין לבין</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr">
+      <c r="I17" s="60" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J17" s="34" t="inlineStr">
+      <c r="J17" s="61" t="inlineStr">
         <is>
           <t>פרק_05_מעברים_וסף_BLOG.svg</t>
         </is>
@@ -1577,7 +1626,7 @@
       <c r="G19" s="15" t="inlineStr"/>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>❌ חסר סקריפט — יש לייצר</t>
+          <t>❌ חסר סקריפט — יש לייצר (גרסת new_beginnings קיימת ב-articles)</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
@@ -1592,53 +1641,53 @@
       </c>
     </row>
     <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="60" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>ביקורת מערכתית
 בית הספר לא נכשל</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="61" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="61" t="inlineStr">
         <is>
           <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_en_blog_20260409_1329.md</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="61" t="inlineStr">
         <is>
           <t>בית הספר לא נכשל — הוא הצליח לעשות בדיוק מה שתוכנן</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="61" t="inlineStr">
         <is>
           <t>שבוע 6</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G20" s="61" t="inlineStr">
         <is>
           <t>חינוך בלתי פורמלי, שייכות, עיצוב אוניברסלי, יזמות חברתית</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H20" s="61" t="inlineStr">
         <is>
           <t>⚠️ קיימת גרסה חדשה — v2 (2007). לבחור לפני פרסום</t>
         </is>
       </c>
-      <c r="I20" s="40" t="inlineStr">
+      <c r="I20" s="60" t="inlineStr">
         <is>
           <t>⚠️ לבחור גרסה</t>
         </is>
       </c>
-      <c r="J20" s="34" t="inlineStr">
+      <c r="J20" s="61" t="inlineStr">
         <is>
           <t>פרק_06_ביקורת_מערכתית_BLOG.svg</t>
         </is>
@@ -1773,53 +1822,53 @@
       </c>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="46" t="inlineStr">
+      <c r="A24" s="62" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>המבנה הוא המסר
 ראובן כהנא</t>
         </is>
       </c>
-      <c r="C24" s="47" t="inlineStr">
+      <c r="C24" s="62" t="inlineStr">
         <is>
           <t>📝 בלוג</t>
         </is>
       </c>
-      <c r="D24" s="48" t="inlineStr">
+      <c r="D24" s="61" t="inlineStr">
         <is>
           <t>פרק_07_המבנה_הוא_המסר_BLOG.md</t>
         </is>
       </c>
-      <c r="E24" s="48" t="inlineStr">
+      <c r="E24" s="61" t="inlineStr">
         <is>
           <t>המבנה הוא המסר: מה שבית הספר לא יכול לעשות — ולמה</t>
         </is>
       </c>
-      <c r="F24" s="47" t="inlineStr">
+      <c r="F24" s="62" t="inlineStr">
         <is>
           <t>שבוע 7</t>
         </is>
       </c>
-      <c r="G24" s="48" t="inlineStr">
+      <c r="G24" s="61" t="inlineStr">
         <is>
           <t>ראובן כהנא, תנועות נוער, מבנה ותוכן, זהות, מדריכים</t>
         </is>
       </c>
-      <c r="H24" s="48" t="inlineStr">
+      <c r="H24" s="61" t="inlineStr">
         <is>
           <t>פרק חדש! על תיאוריית כהנא — המבנה מאפשר זהות</t>
         </is>
       </c>
-      <c r="I24" s="49" t="inlineStr">
+      <c r="I24" s="62" t="inlineStr">
         <is>
           <t>✅ מוכן</t>
         </is>
       </c>
-      <c r="J24" s="50" t="inlineStr">
+      <c r="J24" s="61" t="inlineStr">
         <is>
           <t>פרק_07_המבנה_הוא_המסר_BLOG.svg</t>
         </is>
@@ -1891,7 +1940,7 @@
       <c r="G26" s="53" t="inlineStr"/>
       <c r="H26" s="53" t="inlineStr">
         <is>
-          <t>❌ חסר סקריפט — יש לייצר</t>
+          <t>❌ חסר סקריפט — יש לייצר (מקור: reuven_kahana article קיים)</t>
         </is>
       </c>
       <c r="I26" s="54" t="inlineStr">
@@ -1902,6 +1951,240 @@
       <c r="J26" s="55" t="inlineStr">
         <is>
           <t>❌ חסר עיצוד</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B27" s="63" t="inlineStr">
+        <is>
+          <t>מנהיגות חינוכית
+את מי אנחנו מפתחים?</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>📝 בלוג</t>
+        </is>
+      </c>
+      <c r="D27" s="63" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_blog_20260411_1516.md</t>
+        </is>
+      </c>
+      <c r="E27" s="63" t="inlineStr">
+        <is>
+          <t>את מי בדיוק אנחנו מפתחים כשאנחנו מפתחים מנהיגות?</t>
+        </is>
+      </c>
+      <c r="F27" s="63" t="inlineStr">
+        <is>
+          <t>שבוע 8</t>
+        </is>
+      </c>
+      <c r="G27" s="63" t="inlineStr">
+        <is>
+          <t>מנהיגות נוער, כפר נוער, שייכות, פיתוח מנהיגות</t>
+        </is>
+      </c>
+      <c r="H27" s="63" t="inlineStr">
+        <is>
+          <t>פרק חדש — פוסט בלוג עמוק על מנהיגות ושייכות</t>
+        </is>
+      </c>
+      <c r="I27" s="63" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J27" s="63" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_blog_202604_blog_20260411_1526.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="57" t="n"/>
+      <c r="B28" s="57" t="n"/>
+      <c r="C28" s="57" t="inlineStr">
+        <is>
+          <t>💼 לינקדאין (EN)</t>
+        </is>
+      </c>
+      <c r="D28" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_linkedin_ready.txt</t>
+        </is>
+      </c>
+      <c r="E28" s="57" t="inlineStr">
+        <is>
+          <t>("כל תוכנית מנהיגות שאני מכיר מודדת אותו דבר...")</t>
+        </is>
+      </c>
+      <c r="F28" s="57" t="inlineStr">
+        <is>
+          <t>שבוע 8</t>
+        </is>
+      </c>
+      <c r="G28" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות, כפר נוער, שייכות</t>
+        </is>
+      </c>
+      <c r="H28" s="57" t="inlineStr">
+        <is>
+          <t>גרסה אנגלית</t>
+        </is>
+      </c>
+      <c r="I28" s="57" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J28" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_linkedin_re_linkedin_20260411_1522.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="57" t="n"/>
+      <c r="B29" s="57" t="n"/>
+      <c r="C29" s="57" t="inlineStr">
+        <is>
+          <t>💼 לינקדאין (HE)</t>
+        </is>
+      </c>
+      <c r="D29" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he_linkedin_ready.txt</t>
+        </is>
+      </c>
+      <c r="E29" s="57" t="inlineStr">
+        <is>
+          <t>("יש נוער שנולד עם ניצוץ מנהיגות...")</t>
+        </is>
+      </c>
+      <c r="F29" s="57" t="inlineStr">
+        <is>
+          <t>שבוע 8</t>
+        </is>
+      </c>
+      <c r="G29" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות, כפר נוער, שייכות</t>
+        </is>
+      </c>
+      <c r="H29" s="57" t="inlineStr">
+        <is>
+          <t>גרסה עברית — לבחור בין EN ל-HE</t>
+        </is>
+      </c>
+      <c r="I29" s="57" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J29" s="57" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he_linkedin_re_linkedin_20260410_1739.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="n"/>
+      <c r="B30" s="58" t="n"/>
+      <c r="C30" s="58" t="inlineStr">
+        <is>
+          <t>🎙️ פודקאסט</t>
+        </is>
+      </c>
+      <c r="D30" s="58" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_podcast_script_20260411_1518.md</t>
+        </is>
+      </c>
+      <c r="E30" s="58" t="inlineStr">
+        <is>
+          <t>פרק 8: מי מחליט מי מנהיג?</t>
+        </is>
+      </c>
+      <c r="F30" s="58" t="inlineStr">
+        <is>
+          <t>שבוע 8</t>
+        </is>
+      </c>
+      <c r="G30" s="58" t="inlineStr">
+        <is>
+          <t>מנהיגות, שייכות, כפר נוער</t>
+        </is>
+      </c>
+      <c r="H30" s="58" t="inlineStr">
+        <is>
+          <t>סקריפט ושו-נוטס קיימים (28 דקות)</t>
+        </is>
+      </c>
+      <c r="I30" s="58" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J30" s="58" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_podcast_sho_podcast_20260411_1532.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="57" t="n"/>
+      <c r="B31" s="57" t="inlineStr">
+        <is>
+          <t>🔁 פוסט בונוס
+יזמות חברתית</t>
+        </is>
+      </c>
+      <c r="C31" s="57" t="inlineStr">
+        <is>
+          <t>💼 לינקדאין (בונוס)</t>
+        </is>
+      </c>
+      <c r="D31" s="57" t="inlineStr">
+        <is>
+          <t>בונוס_יזמות_חברתית_LINKEDIN.txt</t>
+        </is>
+      </c>
+      <c r="E31" s="57" t="inlineStr">
+        <is>
+          <t>("בשנה הרביעית בכפר הנוער...")</t>
+        </is>
+      </c>
+      <c r="F31" s="57" t="inlineStr">
+        <is>
+          <t>גמיש</t>
+        </is>
+      </c>
+      <c r="G31" s="57" t="inlineStr">
+        <is>
+          <t>יזמות חברתית, כפר נוער, פדגוגיה</t>
+        </is>
+      </c>
+      <c r="H31" s="57" t="inlineStr">
+        <is>
+          <t>פוסט בונוס על יזמות חברתית — לפרסם בין הפרקים</t>
+        </is>
+      </c>
+      <c r="I31" s="57" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="J31" s="57" t="inlineStr">
+        <is>
+          <t>פרק_06_ביקורת_מערכתית_LINKEDIN.svg</t>
         </is>
       </c>
     </row>
@@ -1920,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2901,6 +3184,2386 @@
         </is>
       </c>
       <c r="F34" s="21" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_en_blog_20260409_2007.md</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>פרק 6 v2 — ביקורת מערכתית (מקור גולמי)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה חדשה</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>מקור ל-פרק_06_ביקורת_מערכתית_BLOG_v2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>reuven_kahana_n_x_reuven_kahana_y_x_non-formal_edu_en_blog_20260409_2053.md</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>פרק 7 — כהנא (מקור גולמי)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה גולמית</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>מקור ל-פרק_07_המבנה_הוא_המסר_BLOG.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_blog_20260411_1516.md</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות חינוכית</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>פרק חדש — 11/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>בונוס_יזמות_חברתית_LINKEDIN.txt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>בונוס — יזמות חברתית</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>פוסט בונוס לפרק 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_linkedin_ready.txt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות (EN)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>גרסה אנגלית</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he_linkedin_ready.txt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות (HE)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>גרסה עברית</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>posts/podcast</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_podcast_script_20260411_1518.md</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות (פודקאסט)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>פודקאסט</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>סקריפט 28 דקות + show notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_blog_202604_blog_20260411_1526.svg</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>פרק 8 — עיצוב בלוג</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_linkedin_re_linkedin_20260411_1522.svg</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>פרק 8 — עיצוב לינקדאין EN</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he_linkedin_re_linkedin_20260410_1739.svg</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>פרק 8 — עיצוב לינקדאין HE</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>designs</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en_podcast_sho_podcast_20260411_1532.svg</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>פרק 8 — עיצוב פודקאסט</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>youth_movements_x_peer_mentorship_x_assessment_and_en.md</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>פרק 1 — שייכות ומדידה</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>youth_movements_x_peer_mentorship_x_assessment_and_en.docx</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>פרק 1 — שייכות ומדידה</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>youth_movements_x_peer_mentorship_x_assessment_and_he.md</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>פרק 1 — שייכות ומדידה</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>youth_movements_x_peer_mentorship_x_assessment_and_he.docx</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>פרק 1 — שייכות ומדידה</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>education_durin_x_education_for_h_x_non-formal_edu_en.md</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>פרק 2 — תקווה ומדידה (סינתזה)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>education_durin_x_education_for_h_x_non-formal_edu_en.docx</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>פרק 2 — תקווה ומדידה (סינתזה)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>education_durin_x_education_for_h_x_non-formal_edu_he.md</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>פרק 2 — תקווה (סינתזה)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>education_durin_x_education_for_h_x_non-formal_edu_he.docx</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>פרק 2 — תקווה (סינתזה)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>education_during_war_and_emergency_israe_en.md</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך בחירום</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>education_during_war_and_emergency_israe_en.docx</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך בחירום</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>education_during_war_and_emergency_israe_he.md</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך בחירום</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>education_during_war_and_emergency_israe_he.docx</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך בחירום</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>education_for_hope_en.md</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך לתקווה</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>education_for_hope_en.docx</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך לתקווה</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>education_for_hope_he.md</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך לתקווה</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>education_for_hope_he.docx</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>פרק 2 — חינוך לתקווה</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>boarding_school_x_hope_theory_and_x_melting_pot_id_en.md</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>פרק 2 — כפר נוער ותקווה (נוסף)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>boarding_school_x_hope_theory_and_x_melting_pot_id_en.docx</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>פרק 2 — כפר נוער ותקווה (נוסף)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_arts-based_non-_x_digital_youth__en.md</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>פרק 3 — מרחב, אומנות, outdoor</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_arts-based_non-_x_digital_youth__en.docx</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>פרק 3 — מרחב, אומנות, outdoor</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_arts-based_non-_x_digital_youth__he.md</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>פרק 3 — מרחב, אומנות, outdoor</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_arts-based_non-_x_digital_youth__he.docx</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>פרק 3 — מרחב, אומנות, outdoor</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_non-formal_educ_x_social_entrepr_en.md</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>פרק 3+6 — outdoor ויזמות</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_non-formal_educ_x_social_entrepr_en.docx</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>פרק 3+6 — outdoor ויזמות</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_non-formal_educ_x_social_entrepr_he.md</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>פרק 3+6 — outdoor ויזמות</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>outdoor_and_adv_x_non-formal_educ_x_social_entrepr_he.docx</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>פרק 3+6 — outdoor ויזמות</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>digital_youth_w_x_digital_youth_w_x_arts-based_non_en.md</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>פרק 4 — נוער דיגיטלי</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>digital_youth_w_x_digital_youth_w_x_arts-based_non_en.docx</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>פרק 4 — נוער דיגיטלי</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>digital_youth_w_x_digital_youth_w_x_arts-based_non_he.md</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>פרק 4 — נוער דיגיטלי</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>digital_youth_w_x_digital_youth_w_x_arts-based_non_he.docx</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>פרק 4 — נוער דיגיטלי</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>new_beginnings__x_fresh_start_eff_x_threshold_conc_en.md</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>פרק 5 — מעברים וסף</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>new_beginnings__x_fresh_start_eff_x_threshold_conc_en.docx</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>פרק 5 — מעברים וסף</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_en.md</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת ויזמות חברתית</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_en.docx</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת ויזמות חברתית</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_he.md</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת ויזמות חברתית</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>non-formal_educ_x_social_entrepre_x_non-formal_edu_he.docx</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת ויזמות חברתית</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>critique_of_non_x_emotional_and_s_x_arts-based_non_en.md</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת מבנית + גוף</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>critique_of_non_x_emotional_and_s_x_arts-based_non_en.docx</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>פרק 6 — ביקורת מבנית + גוף</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>reuven_kahana_n_x_reuven_kahana_y_x_non-formal_edu_en.md</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>פרק 7 — ראובן כהנא (מקור)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>reuven_kahana_n_x_reuven_kahana_y_x_non-formal_edu_en.docx</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>פרק 7 — ראובן כהנא (מקור)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>reuven_kahana_n_x_reuven_kahana_y_x_non-formal_edu_he.md</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>פרק 7 — ראובן כהנא (מקור)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>reuven_kahana_n_x_reuven_kahana_y_x_non-formal_edu_he.docx</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>פרק 7 — ראובן כהנא (מקור)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en.md</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות חינוכית</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_en.docx</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות חינוכית</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he.md</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות חינוכית</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>מנהיגות_חינוכית_he.docx</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות חינוכית</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>non-formal_education.md</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: עברית/אנגלית</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>non-formal_education.docx</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: עברית/אנגלית</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>non-formal_education_en.md</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>non-formal_education_en.docx</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>non-formal_education_he.md</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>non-formal_education_he.docx</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>מבוא — חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>non-formal_education_system_en.md</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>מבוא — מערכת חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>non-formal_education_system_en.docx</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>מבוא — מערכת חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: EN</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>non-formal_education_system_he.md</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>מבוא — מערכת חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>📚 מקור</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>non-formal_education_system_he.docx</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>מבוא — מערכת חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>מאמר אקדמי</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>📚 מקור (.docx)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>מאמר מקור | שפה: HE</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>output/</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>svg_belonging.svg</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>פרק 1 — שייכות</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>SVG עצמאי ב-output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>output/</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>podcast_ch1_who_decides.svg</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>פרק 1 — פודקאסט</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>SVG עצמאי ב-output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>output/</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>linkedin_cover_kahana.svg</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>פרק 7 — כהנא</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>SVG עצמאי ב-output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>output/</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>linkedin_quiet_leader.svg</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>פרק 8 — מנהיגות</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>עיצוב</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>✅ מוכן</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>SVG עצמאי ב-output/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>posts/</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>education_for_hope_en_podcast_script_20260407_1028.md</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>פרק 2 — תקווה (גרסה מוקדמת)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>פודקאסט</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה מוקדמת</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>ב-posts/ root — יכול לשמש פרק 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>posts/</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>education_during_war_and_emergency_israe_en_podcast_script_20260407_1040.md</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>פרק 2 — חירום (גרסה מוקדמת)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>פודקאסט</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה מוקדמת</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>ב-posts/ root</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>posts/</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>non-formal_education_en_podcast_script_20260406_1535.md</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>מבוא — פודקאסט (גרסה מוקדמת)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>פודקאסט</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה מוקדמת</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>ב-posts/ root — teaser/מבוא</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>posts/</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>non-formal_education_system_en_podcast_script_20260407_0949.md</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>מבוא מערכת — פודקאסט</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>פודקאסט</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה מוקדמת</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>ב-posts/ root</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Fix chat crash on CLIUnavailable + budget pre-check + Agent 6 budget timing
</commit_message>
<xml_diff>
--- a/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
+++ b/לוח_פרסום_חינוך_בלתי_פורמלי.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -605,6 +605,9 @@
     <xf numFmtId="0" fontId="0" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -970,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2807,7 +2810,6 @@
       <c r="I46" s="54" t="n"/>
       <c r="J46" s="55" t="n"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="56" t="inlineStr">
         <is>
@@ -2945,7 +2947,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="56" t="inlineStr">
         <is>
@@ -3087,7 +3088,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
     <row r="56">
       <c r="A56" s="80" t="inlineStr">
         <is>
@@ -3511,7 +3511,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="88" t="inlineStr">
         <is>
@@ -3645,7 +3644,6 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
     <row r="70">
       <c r="A70" s="88" t="inlineStr">
         <is>
@@ -3775,7 +3773,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="A74" s="91" t="inlineStr">
         <is>
@@ -3902,6 +3899,143 @@
       <c r="J76" s="90" t="inlineStr">
         <is>
           <t>פרק_20_שייכות_חברתית_PODCAST.svg</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="93" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B78" s="93" t="inlineStr">
+        <is>
+          <t>זהות מקצועית במעבר תפקידים
+כשהמוסד זוכר אותך יותר ממך</t>
+        </is>
+      </c>
+      <c r="C78" s="93" t="inlineStr">
+        <is>
+          <t>📝 בלוג</t>
+        </is>
+      </c>
+      <c r="D78" s="93" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_blog_20260514_0713.md</t>
+        </is>
+      </c>
+      <c r="E78" s="93" t="inlineStr">
+        <is>
+          <t>כשהמוסד זוכר אותך יותר ממך — על חזרת בוגרים ותסמונת מתחזה</t>
+        </is>
+      </c>
+      <c r="F78" s="93" t="inlineStr">
+        <is>
+          <t>טרם נקבע</t>
+        </is>
+      </c>
+      <c r="G78" s="93" t="inlineStr">
+        <is>
+          <t>זהות מקצועית, מעבר תפקידים, תנועות נוער, מנהיגות חינוכית, תסמונת מתחזה</t>
+        </is>
+      </c>
+      <c r="H78" s="93" t="inlineStr">
+        <is>
+          <t>שתי גרסאות בלוג (13/05 ו-14/05). גרסה 14/05 = מומלצת. גרסה 13/05: "הכותרת על הדלת השתנתה"</t>
+        </is>
+      </c>
+      <c r="I78" s="93" t="inlineStr">
+        <is>
+          <t>⚠️ דרפט</t>
+        </is>
+      </c>
+      <c r="J78" s="93" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="94" t="n"/>
+      <c r="B79" s="94" t="n"/>
+      <c r="C79" s="94" t="inlineStr">
+        <is>
+          <t>💼 לינקדאין</t>
+        </is>
+      </c>
+      <c r="D79" s="94" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_ready_20260514_0706.txt</t>
+        </is>
+      </c>
+      <c r="E79" s="94" t="inlineStr">
+        <is>
+          <t>"מתי הרגשת בפעם האחרונה כמו מתחזה — לא בהתחלה, אלא דווקא אחרי שעלית תפקיד?"</t>
+        </is>
+      </c>
+      <c r="F79" s="94" t="inlineStr">
+        <is>
+          <t>טרם נקבע</t>
+        </is>
+      </c>
+      <c r="G79" s="94" t="inlineStr">
+        <is>
+          <t>זהות, מנהיגות, מעבר תפקידים, חינוך בלתי פורמלי</t>
+        </is>
+      </c>
+      <c r="H79" s="94" t="inlineStr">
+        <is>
+          <t>גרסה B גם זמינה: linkedin_B_20260514_0706 | גרסה ראשונה: 13/05 | גרסת ready: 14/05</t>
+        </is>
+      </c>
+      <c r="I79" s="94" t="inlineStr">
+        <is>
+          <t>⚠️ דרפט</t>
+        </is>
+      </c>
+      <c r="J79" s="94" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="95" t="n"/>
+      <c r="B80" s="95" t="n"/>
+      <c r="C80" s="95" t="inlineStr">
+        <is>
+          <t>🎙️ פודקאסט</t>
+        </is>
+      </c>
+      <c r="D80" s="95" t="inlineStr">
+        <is>
+          <t>❌ חסר</t>
+        </is>
+      </c>
+      <c r="E80" s="95" t="inlineStr">
+        <is>
+          <t>פרק 21: עדיין לא נוצר</t>
+        </is>
+      </c>
+      <c r="F80" s="95" t="inlineStr">
+        <is>
+          <t>טרם נקבע</t>
+        </is>
+      </c>
+      <c r="G80" s="95" t="n"/>
+      <c r="H80" s="95" t="inlineStr">
+        <is>
+          <t>❌ חסר סקריפט — יש לייצר</t>
+        </is>
+      </c>
+      <c r="I80" s="95" t="inlineStr">
+        <is>
+          <t>❌ חסר</t>
+        </is>
+      </c>
+      <c r="J80" s="95" t="inlineStr">
+        <is>
+          <t>❌ חסר עיצוב</t>
         </is>
       </c>
     </row>
@@ -3920,7 +4054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F324"/>
+  <dimension ref="A1:F332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14115,6 +14249,262 @@
       <c r="F324" s="92" t="inlineStr">
         <is>
           <t>נוצר 10/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_blog_20260514_0713.md</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>✅ מומלץ לפרסום</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>"כשהמוסד זוכר אותך יותר ממך" — גרסה סופית 14/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>posts/blog</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_blog_20260513_1858.md</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>בלוג</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה ראשונה</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>"הכותרת על הדלת השתנתה. הזהות לא." — 13/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_ready_20260514_0706.txt</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>✅ מוכן לפרסום</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>גרסה ready 14/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_20260514_0706.txt</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>⚠️ דרפט</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>14/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_B_20260514_0706.txt</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה B</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>14/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_ready_20260513_1846.txt</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה ראשונה ready</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>13/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_20260513_1846.txt</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>⚠️ דרפט</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>13/05</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>posts/linkedin</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>psychosocial_transit_x_identity_renegotiati_x_peer_legacy_tr_he_linkedin_B_20260513_1846.txt</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>פרק 21 — זהות מקצועית במעבר תפקידים</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>לינקדאין</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>⚠️ גרסה B</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>13/05</t>
         </is>
       </c>
     </row>
@@ -14132,7 +14522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14252,7 +14642,8 @@
       <c r="B10" s="30" t="inlineStr">
         <is>
           <t>פרקים 2, 3, 5, 7 — אין סקריפט פודקאסט. יש ליצור לפני הפרסום.
-פרק 12 ו-17 ✅ הושלמו (04/05/2026).</t>
+פרק 12 ו-17 ✅ הושלמו (04/05/2026).
+פרק 21 — זהות מקצועית במעבר תפקידים: אין סקריפט פודקאסט, אין עיצובים. נוסף 17/05/2026.</t>
         </is>
       </c>
     </row>
@@ -14281,6 +14672,19 @@
           <t>כל קבצי ה-SVG נמצאים בתיקייה:
 output/designs/
 הקבצים הממוספרים (פרק_01_...) הם הגרסאות הסופיות לפרסום.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>פרק 21</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>זהות מקצועית במעבר תפקידים
+→ כשהמדריך הופך לראש צוות, והמוסד לא בנה לו גשר. על תסמונת מתחזה כמנגנון מוסדי, חזרת בוגרים, ומסירת מורשת עמיתים. שני פוסטי בלוג נכתבו (13/05, 14/05). חסרים: סקריפט פודקאסט + עיצובים (3 פלטפורמות). נוסף 17/05/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>